<commit_message>
added logic of calculation of full length of compressor
</commit_message>
<xml_diff>
--- a/results/Начальные_данные.xlsx
+++ b/results/Начальные_данные.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.433333</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.366666</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">

</xml_diff>